<commit_message>
add extension IsDeleted 9ef355b6f3e81ec5270d311474b08990da3a85a1
</commit_message>
<xml_diff>
--- a/add-ext-deleted/ig/StructureDefinition-pdsm-submissionset-comprehensive.xlsx
+++ b/add-ext-deleted/ig/StructureDefinition-pdsm-submissionset-comprehensive.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$65</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2332" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2368" uniqueCount="459">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-29T08:38:17+00:00</t>
+    <t>2026-09-30T10:37:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -765,6 +765,22 @@
   </si>
   <si>
     <t>statut : [1..1] Code</t>
+  </si>
+  <si>
+    <t>List.extension:isDeleted</t>
+  </si>
+  <si>
+    <t>isDeleted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://interop.esante.gouv.fr/ig/fhir/pdsm/StructureDefinition/pdsm-ext-is-deleted}
+</t>
+  </si>
+  <si>
+    <t>Extension définie par ce volet pour distinguer les lots de soumission supprimés. Suppression logique pas physique.</t>
+  </si>
+  <si>
+    <t>Extension définie par le volet ANS "Volet Partage de documents de santé en mobilité" sur les ressources List et DocumentReference pour distinguer les lots de soumission et les fiches supprimées. A noter que la suppression est logique et pas physique.</t>
   </si>
   <si>
     <t>List.extension:PDSmintendedRecipient</t>
@@ -1757,7 +1773,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN64"/>
+  <dimension ref="A1:AN65"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="39.5859375" customWidth="true" bestFit="true"/>
@@ -4641,7 +4657,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
         <v>239</v>
       </c>
@@ -4659,10 +4675,10 @@
         <v>78</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>80</v>
@@ -4743,7 +4759,7 @@
         <v>118</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>80</v>
+        <v>238</v>
       </c>
       <c r="AL26" t="s" s="2">
         <v>80</v>
@@ -4755,14 +4771,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="27" hidden="true">
+    <row r="27">
       <c r="A27" t="s" s="2">
         <v>244</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>204</v>
-      </c>
-      <c r="C27" s="2"/>
+        <v>190</v>
+      </c>
+      <c r="C27" t="s" s="2">
+        <v>245</v>
+      </c>
       <c r="D27" t="s" s="2">
         <v>80</v>
       </c>
@@ -4771,10 +4789,10 @@
         <v>78</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>80</v>
@@ -4783,13 +4801,13 @@
         <v>80</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>103</v>
+        <v>246</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>104</v>
+        <v>247</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>105</v>
+        <v>248</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4840,19 +4858,19 @@
         <v>80</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>106</v>
+        <v>194</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>80</v>
@@ -4861,7 +4879,7 @@
         <v>80</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>80</v>
@@ -4869,10 +4887,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4883,7 +4901,7 @@
         <v>78</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>80</v>
@@ -4895,13 +4913,13 @@
         <v>80</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4940,31 +4958,31 @@
         <v>80</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="AC28" t="s" s="2">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="AD28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AK28" t="s" s="2">
         <v>80</v>
@@ -4973,7 +4991,7 @@
         <v>80</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>80</v>
@@ -4981,10 +4999,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4992,10 +5010,10 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>80</v>
@@ -5007,24 +5025,22 @@
         <v>80</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>209</v>
+        <v>192</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>210</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>211</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
-        <v>247</v>
+        <v>80</v>
       </c>
       <c r="S29" t="s" s="2">
         <v>80</v>
@@ -5054,31 +5070,31 @@
         <v>80</v>
       </c>
       <c r="AB29" t="s" s="2">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="AC29" t="s" s="2">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="AD29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE29" t="s" s="2">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>213</v>
+        <v>117</v>
       </c>
       <c r="AG29" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>80</v>
@@ -5087,7 +5103,7 @@
         <v>80</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>189</v>
+        <v>80</v>
       </c>
       <c r="AN29" t="s" s="2">
         <v>80</v>
@@ -5095,10 +5111,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5106,7 +5122,7 @@
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G30" t="s" s="2">
         <v>89</v>
@@ -5121,22 +5137,24 @@
         <v>80</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>249</v>
+        <v>131</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>210</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>211</v>
+      </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q30" s="2"/>
       <c r="R30" t="s" s="2">
-        <v>80</v>
+        <v>252</v>
       </c>
       <c r="S30" t="s" s="2">
         <v>80</v>
@@ -5178,10 +5196,10 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="AG30" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="AH30" t="s" s="2">
         <v>89</v>
@@ -5190,7 +5208,7 @@
         <v>80</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>80</v>
@@ -5207,10 +5225,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5221,25 +5239,25 @@
         <v>78</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>110</v>
+        <v>254</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>192</v>
+        <v>217</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>193</v>
+        <v>218</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5290,19 +5308,19 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>251</v>
+        <v>220</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>80</v>
@@ -5311,7 +5329,7 @@
         <v>80</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>80</v>
+        <v>189</v>
       </c>
       <c r="AN31" t="s" s="2">
         <v>80</v>
@@ -5319,10 +5337,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5333,25 +5351,25 @@
         <v>78</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I32" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="J32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>253</v>
+        <v>110</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>254</v>
+        <v>192</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>255</v>
+        <v>193</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5390,17 +5408,19 @@
         <v>80</v>
       </c>
       <c r="AB32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF32" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="AC32" s="2"/>
-      <c r="AD32" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE32" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AF32" t="s" s="2">
-        <v>252</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5412,31 +5432,29 @@
         <v>80</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN32" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" hidden="true">
+      <c r="A33" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="AM32" t="s" s="2">
-        <v>258</v>
-      </c>
-      <c r="AN32" t="s" s="2">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="2">
-        <v>260</v>
-      </c>
       <c r="B33" t="s" s="2">
-        <v>252</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>261</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
         <v>80</v>
       </c>
@@ -5445,10 +5463,10 @@
         <v>78</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H33" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="I33" t="s" s="2">
         <v>80</v>
@@ -5457,13 +5475,13 @@
         <v>80</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5502,19 +5520,17 @@
         <v>80</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC33" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="AC33" s="2"/>
       <c r="AD33" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5529,16 +5545,16 @@
         <v>101</v>
       </c>
       <c r="AK33" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL33" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="AM33" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="AN33" t="s" s="2">
         <v>264</v>
-      </c>
-      <c r="AL33" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM33" t="s" s="2">
-        <v>258</v>
-      </c>
-      <c r="AN33" t="s" s="2">
-        <v>259</v>
       </c>
     </row>
     <row r="34">
@@ -5546,7 +5562,7 @@
         <v>265</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C34" t="s" s="2">
         <v>266</v>
@@ -5559,7 +5575,7 @@
         <v>78</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>90</v>
@@ -5577,7 +5593,7 @@
         <v>268</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5628,7 +5644,7 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5649,10 +5665,10 @@
         <v>80</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="35">
@@ -5660,40 +5676,40 @@
         <v>270</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>270</v>
-      </c>
-      <c r="C35" s="2"/>
+        <v>257</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>271</v>
+      </c>
       <c r="D35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>90</v>
       </c>
       <c r="I35" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>166</v>
+        <v>272</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>272</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>273</v>
-      </c>
+        <v>260</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>80</v>
@@ -5703,7 +5719,7 @@
         <v>80</v>
       </c>
       <c r="S35" t="s" s="2">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="T35" t="s" s="2">
         <v>80</v>
@@ -5718,13 +5734,13 @@
         <v>80</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>275</v>
+        <v>80</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>276</v>
+        <v>80</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>277</v>
+        <v>80</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>80</v>
@@ -5742,13 +5758,13 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>80</v>
@@ -5757,24 +5773,24 @@
         <v>101</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>238</v>
+        <v>274</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>278</v>
+        <v>80</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>280</v>
+        <v>264</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5800,17 +5816,15 @@
         <v>166</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>284</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>285</v>
-      </c>
+        <v>278</v>
+      </c>
+      <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>80</v>
       </c>
@@ -5819,7 +5833,7 @@
         <v>80</v>
       </c>
       <c r="S36" t="s" s="2">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="T36" t="s" s="2">
         <v>80</v>
@@ -5834,31 +5848,31 @@
         <v>80</v>
       </c>
       <c r="X36" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="Y36" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="Z36" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="AA36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF36" t="s" s="2">
         <v>275</v>
-      </c>
-      <c r="Y36" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="Z36" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="AA36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF36" t="s" s="2">
-        <v>281</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>89</v>
@@ -5873,24 +5887,24 @@
         <v>101</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>80</v>
+        <v>238</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>291</v>
+        <v>285</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5898,7 +5912,7 @@
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G37" t="s" s="2">
         <v>89</v>
@@ -5907,23 +5921,25 @@
         <v>90</v>
       </c>
       <c r="I37" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="J37" t="s" s="2">
         <v>90</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>103</v>
+        <v>166</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>294</v>
-      </c>
-      <c r="N37" s="2"/>
+        <v>288</v>
+      </c>
+      <c r="N37" t="s" s="2">
+        <v>289</v>
+      </c>
       <c r="O37" t="s" s="2">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>80</v>
@@ -5933,10 +5949,10 @@
         <v>80</v>
       </c>
       <c r="S37" t="s" s="2">
-        <v>80</v>
+        <v>291</v>
       </c>
       <c r="T37" t="s" s="2">
-        <v>296</v>
+        <v>80</v>
       </c>
       <c r="U37" t="s" s="2">
         <v>80</v>
@@ -5948,13 +5964,13 @@
         <v>80</v>
       </c>
       <c r="X37" t="s" s="2">
-        <v>80</v>
+        <v>280</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>80</v>
+        <v>292</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>80</v>
+        <v>293</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>80</v>
@@ -5972,10 +5988,10 @@
         <v>80</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="AG37" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="AH37" t="s" s="2">
         <v>89</v>
@@ -5987,24 +6003,24 @@
         <v>101</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>297</v>
+        <v>80</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>80</v>
+        <v>296</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6012,7 +6028,7 @@
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G38" t="s" s="2">
         <v>89</v>
@@ -6027,19 +6043,17 @@
         <v>90</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>216</v>
+        <v>103</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>303</v>
-      </c>
+        <v>299</v>
+      </c>
+      <c r="N38" s="2"/>
       <c r="O38" t="s" s="2">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>80</v>
@@ -6049,10 +6063,10 @@
         <v>80</v>
       </c>
       <c r="S38" t="s" s="2">
-        <v>305</v>
+        <v>80</v>
       </c>
       <c r="T38" t="s" s="2">
-        <v>80</v>
+        <v>301</v>
       </c>
       <c r="U38" t="s" s="2">
         <v>80</v>
@@ -6064,11 +6078,13 @@
         <v>80</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>275</v>
-      </c>
-      <c r="Y38" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y38" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z38" t="s" s="2">
-        <v>306</v>
+        <v>80</v>
       </c>
       <c r="AA38" t="s" s="2">
         <v>80</v>
@@ -6086,7 +6102,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -6101,24 +6117,24 @@
         <v>101</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>80</v>
+        <v>302</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>309</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6141,19 +6157,19 @@
         <v>90</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>311</v>
+        <v>216</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="O39" t="s" s="2">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>80</v>
@@ -6163,7 +6179,7 @@
         <v>80</v>
       </c>
       <c r="S39" t="s" s="2">
-        <v>80</v>
+        <v>310</v>
       </c>
       <c r="T39" t="s" s="2">
         <v>80</v>
@@ -6178,13 +6194,11 @@
         <v>80</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y39" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>280</v>
+      </c>
+      <c r="Y39" s="2"/>
       <c r="Z39" t="s" s="2">
-        <v>80</v>
+        <v>311</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>80</v>
@@ -6202,7 +6216,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -6217,24 +6231,24 @@
         <v>101</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>316</v>
+        <v>80</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
-    <row r="40" hidden="true">
+    <row r="40">
       <c r="A40" t="s" s="2">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6242,31 +6256,35 @@
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="N40" s="2"/>
-      <c r="O40" s="2"/>
+        <v>318</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="O40" t="s" s="2">
+        <v>320</v>
+      </c>
       <c r="P40" t="s" s="2">
         <v>80</v>
       </c>
@@ -6314,7 +6332,7 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6329,24 +6347,24 @@
         <v>101</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>80</v>
+        <v>321</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>107</v>
+        <v>322</v>
       </c>
       <c r="AM40" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="AN40" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="AN40" t="s" s="2">
+    </row>
+    <row r="41" hidden="true">
+      <c r="A41" t="s" s="2">
         <v>325</v>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s" s="2">
-        <v>326</v>
-      </c>
       <c r="B41" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6354,35 +6372,31 @@
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>328</v>
       </c>
-      <c r="M41" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="O41" t="s" s="2">
-        <v>331</v>
-      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>80</v>
       </c>
@@ -6430,7 +6444,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6445,28 +6459,28 @@
         <v>101</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>333</v>
+        <v>107</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>337</v>
+        <v>80</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6485,19 +6499,19 @@
         <v>90</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="O42" t="s" s="2">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>80</v>
@@ -6546,7 +6560,7 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6561,56 +6575,60 @@
         <v>101</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>80</v>
+        <v>337</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>345</v>
+        <v>340</v>
       </c>
     </row>
-    <row r="43" hidden="true">
+    <row r="43">
       <c r="A43" t="s" s="2">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>80</v>
+        <v>342</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G43" t="s" s="2">
         <v>89</v>
       </c>
       <c r="H43" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>103</v>
+        <v>343</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>104</v>
+        <v>344</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
+        <v>345</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="O43" t="s" s="2">
+        <v>347</v>
+      </c>
       <c r="P43" t="s" s="2">
         <v>80</v>
       </c>
@@ -6658,7 +6676,7 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>106</v>
+        <v>341</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6670,38 +6688,38 @@
         <v>80</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>80</v>
+        <v>348</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>107</v>
+        <v>349</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>80</v>
+        <v>350</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>80</v>
@@ -6713,17 +6731,15 @@
         <v>80</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>113</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>80</v>
@@ -6760,31 +6776,31 @@
         <v>80</v>
       </c>
       <c r="AB44" t="s" s="2">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AK44" t="s" s="2">
         <v>80</v>
@@ -6801,23 +6817,21 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="C45" t="s" s="2">
-        <v>349</v>
-      </c>
+        <v>352</v>
+      </c>
+      <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>80</v>
@@ -6829,15 +6843,17 @@
         <v>80</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>350</v>
+        <v>110</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>351</v>
+        <v>111</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="N45" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>113</v>
+      </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>80</v>
@@ -6874,16 +6890,16 @@
         <v>80</v>
       </c>
       <c r="AB45" t="s" s="2">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="AC45" t="s" s="2">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="AD45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE45" t="s" s="2">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="AF45" t="s" s="2">
         <v>117</v>
@@ -6901,13 +6917,13 @@
         <v>118</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>353</v>
+        <v>80</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>80</v>
@@ -6915,12 +6931,14 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="C46" t="s" s="2">
         <v>354</v>
       </c>
-      <c r="B46" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
         <v>80</v>
       </c>
@@ -6941,13 +6959,13 @@
         <v>80</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>103</v>
+        <v>355</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>104</v>
+        <v>356</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>105</v>
+        <v>357</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -6998,28 +7016,28 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>80</v>
+        <v>358</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>80</v>
@@ -7027,10 +7045,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7041,7 +7059,7 @@
         <v>78</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>80</v>
@@ -7053,13 +7071,13 @@
         <v>80</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7098,31 +7116,31 @@
         <v>80</v>
       </c>
       <c r="AB47" t="s" s="2">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="AC47" t="s" s="2">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="AD47" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE47" t="s" s="2">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AK47" t="s" s="2">
         <v>80</v>
@@ -7131,7 +7149,7 @@
         <v>80</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>80</v>
@@ -7139,10 +7157,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7150,10 +7168,10 @@
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>80</v>
@@ -7165,24 +7183,22 @@
         <v>80</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>209</v>
+        <v>192</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>210</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>211</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q48" s="2"/>
       <c r="R48" t="s" s="2">
-        <v>360</v>
+        <v>80</v>
       </c>
       <c r="S48" t="s" s="2">
         <v>80</v>
@@ -7212,31 +7228,31 @@
         <v>80</v>
       </c>
       <c r="AB48" t="s" s="2">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="AC48" t="s" s="2">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="AD48" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE48" t="s" s="2">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>213</v>
+        <v>117</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ48" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AK48" t="s" s="2">
         <v>80</v>
@@ -7245,7 +7261,7 @@
         <v>80</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>189</v>
+        <v>80</v>
       </c>
       <c r="AN48" t="s" s="2">
         <v>80</v>
@@ -7253,10 +7269,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7279,22 +7295,24 @@
         <v>80</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>363</v>
+        <v>131</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="N49" s="2"/>
+        <v>210</v>
+      </c>
+      <c r="N49" t="s" s="2">
+        <v>211</v>
+      </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q49" s="2"/>
       <c r="R49" t="s" s="2">
-        <v>80</v>
+        <v>365</v>
       </c>
       <c r="S49" t="s" s="2">
         <v>80</v>
@@ -7336,10 +7354,10 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="AG49" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="AH49" t="s" s="2">
         <v>89</v>
@@ -7348,7 +7366,7 @@
         <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>80</v>
@@ -7365,10 +7383,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7376,7 +7394,7 @@
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G50" t="s" s="2">
         <v>89</v>
@@ -7388,20 +7406,18 @@
         <v>80</v>
       </c>
       <c r="J50" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>103</v>
+        <v>368</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>365</v>
+        <v>217</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>366</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>367</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
         <v>80</v>
@@ -7450,7 +7466,7 @@
         <v>80</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>368</v>
+        <v>220</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>78</v>
@@ -7459,7 +7475,7 @@
         <v>89</v>
       </c>
       <c r="AI50" t="s" s="2">
-        <v>369</v>
+        <v>80</v>
       </c>
       <c r="AJ50" t="s" s="2">
         <v>101</v>
@@ -7479,10 +7495,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7505,16 +7521,16 @@
         <v>90</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>131</v>
+        <v>103</v>
       </c>
       <c r="L51" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="M51" t="s" s="2">
         <v>371</v>
       </c>
-      <c r="M51" t="s" s="2">
+      <c r="N51" t="s" s="2">
         <v>372</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>373</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
@@ -7540,40 +7556,40 @@
         <v>80</v>
       </c>
       <c r="X51" t="s" s="2">
-        <v>148</v>
+        <v>80</v>
       </c>
       <c r="Y51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF51" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="AG51" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH51" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI51" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>375</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>376</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>80</v>
       </c>
       <c r="AJ51" t="s" s="2">
         <v>101</v>
@@ -7593,10 +7609,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7619,16 +7635,16 @@
         <v>90</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>253</v>
+        <v>131</v>
       </c>
       <c r="L52" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="M52" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="N52" t="s" s="2">
         <v>378</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>379</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>380</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -7654,13 +7670,13 @@
         <v>80</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="Y52" t="s" s="2">
-        <v>80</v>
+        <v>379</v>
       </c>
       <c r="Z52" t="s" s="2">
-        <v>80</v>
+        <v>380</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>80</v>
@@ -7699,7 +7715,7 @@
         <v>80</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>382</v>
+        <v>189</v>
       </c>
       <c r="AN52" t="s" s="2">
         <v>80</v>
@@ -7707,10 +7723,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7733,16 +7749,16 @@
         <v>90</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>103</v>
+        <v>258</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>383</v>
+      </c>
+      <c r="M53" t="s" s="2">
         <v>384</v>
       </c>
-      <c r="M53" t="s" s="2">
+      <c r="N53" t="s" s="2">
         <v>385</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>386</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -7792,7 +7808,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7813,7 +7829,7 @@
         <v>80</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>189</v>
+        <v>387</v>
       </c>
       <c r="AN53" t="s" s="2">
         <v>80</v>
@@ -7835,7 +7851,7 @@
         <v>78</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>80</v>
@@ -7844,10 +7860,10 @@
         <v>80</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>216</v>
+        <v>103</v>
       </c>
       <c r="L54" t="s" s="2">
         <v>389</v>
@@ -7858,9 +7874,7 @@
       <c r="N54" t="s" s="2">
         <v>391</v>
       </c>
-      <c r="O54" t="s" s="2">
-        <v>392</v>
-      </c>
+      <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
         <v>80</v>
       </c>
@@ -7884,13 +7898,13 @@
         <v>80</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>170</v>
+        <v>80</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>393</v>
+        <v>80</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>394</v>
+        <v>80</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>80</v>
@@ -7908,7 +7922,7 @@
         <v>80</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -7926,10 +7940,10 @@
         <v>80</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>395</v>
+        <v>189</v>
       </c>
       <c r="AN54" t="s" s="2">
         <v>80</v>
@@ -7937,10 +7951,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -7951,7 +7965,7 @@
         <v>78</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>80</v>
@@ -7963,16 +7977,20 @@
         <v>80</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="L55" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="M55" t="s" s="2">
+        <v>395</v>
+      </c>
+      <c r="N55" t="s" s="2">
+        <v>396</v>
+      </c>
+      <c r="O55" t="s" s="2">
         <v>397</v>
       </c>
-      <c r="L55" t="s" s="2">
-        <v>398</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>399</v>
-      </c>
-      <c r="N55" s="2"/>
-      <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
         <v>80</v>
       </c>
@@ -7996,13 +8014,13 @@
         <v>80</v>
       </c>
       <c r="X55" t="s" s="2">
-        <v>80</v>
+        <v>170</v>
       </c>
       <c r="Y55" t="s" s="2">
-        <v>80</v>
+        <v>398</v>
       </c>
       <c r="Z55" t="s" s="2">
-        <v>80</v>
+        <v>399</v>
       </c>
       <c r="AA55" t="s" s="2">
         <v>80</v>
@@ -8020,13 +8038,13 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH55" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI55" t="s" s="2">
         <v>80</v>
@@ -8035,13 +8053,13 @@
         <v>101</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AM55" t="s" s="2">
         <v>400</v>
-      </c>
-      <c r="AL55" t="s" s="2">
-        <v>401</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>402</v>
       </c>
       <c r="AN55" t="s" s="2">
         <v>80</v>
@@ -8049,10 +8067,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8063,7 +8081,7 @@
         <v>78</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H56" t="s" s="2">
         <v>80</v>
@@ -8075,17 +8093,15 @@
         <v>80</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>402</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="M56" t="s" s="2">
         <v>404</v>
       </c>
-      <c r="L56" t="s" s="2">
-        <v>405</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>406</v>
-      </c>
-      <c r="N56" t="s" s="2">
-        <v>407</v>
-      </c>
+      <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>80</v>
@@ -8134,7 +8150,7 @@
         <v>80</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>78</v>
@@ -8143,19 +8159,19 @@
         <v>79</v>
       </c>
       <c r="AI56" t="s" s="2">
-        <v>408</v>
+        <v>80</v>
       </c>
       <c r="AJ56" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>80</v>
+        <v>405</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>80</v>
+        <v>406</v>
       </c>
       <c r="AM56" t="s" s="2">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="AN56" t="s" s="2">
         <v>80</v>
@@ -8163,10 +8179,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8177,7 +8193,7 @@
         <v>78</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>80</v>
@@ -8189,15 +8205,17 @@
         <v>80</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>103</v>
+        <v>409</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>104</v>
+        <v>410</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N57" s="2"/>
+        <v>411</v>
+      </c>
+      <c r="N57" t="s" s="2">
+        <v>412</v>
+      </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>80</v>
@@ -8246,19 +8264,19 @@
         <v>80</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>106</v>
+        <v>408</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH57" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI57" t="s" s="2">
-        <v>80</v>
+        <v>413</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="AK57" t="s" s="2">
         <v>80</v>
@@ -8267,7 +8285,7 @@
         <v>80</v>
       </c>
       <c r="AM57" t="s" s="2">
-        <v>107</v>
+        <v>414</v>
       </c>
       <c r="AN57" t="s" s="2">
         <v>80</v>
@@ -8275,21 +8293,21 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G58" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H58" t="s" s="2">
         <v>80</v>
@@ -8301,17 +8319,15 @@
         <v>80</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>113</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
         <v>80</v>
@@ -8360,19 +8376,19 @@
         <v>80</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH58" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI58" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>80</v>
@@ -8389,14 +8405,14 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
-        <v>413</v>
+        <v>109</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
@@ -8409,26 +8425,24 @@
         <v>80</v>
       </c>
       <c r="I59" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K59" t="s" s="2">
         <v>110</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>414</v>
+        <v>111</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>415</v>
+        <v>112</v>
       </c>
       <c r="N59" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="O59" t="s" s="2">
-        <v>416</v>
-      </c>
+      <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
         <v>80</v>
       </c>
@@ -8476,7 +8490,7 @@
         <v>80</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>417</v>
+        <v>117</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
@@ -8497,7 +8511,7 @@
         <v>80</v>
       </c>
       <c r="AM59" t="s" s="2">
-        <v>189</v>
+        <v>107</v>
       </c>
       <c r="AN59" t="s" s="2">
         <v>80</v>
@@ -8505,33 +8519,33 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>80</v>
+        <v>418</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I60" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="J60" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>216</v>
+        <v>110</v>
       </c>
       <c r="L60" t="s" s="2">
         <v>419</v>
@@ -8540,10 +8554,10 @@
         <v>420</v>
       </c>
       <c r="N60" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="O60" t="s" s="2">
         <v>421</v>
-      </c>
-      <c r="O60" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="P60" t="s" s="2">
         <v>80</v>
@@ -8568,13 +8582,13 @@
         <v>80</v>
       </c>
       <c r="X60" t="s" s="2">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="Y60" t="s" s="2">
-        <v>423</v>
+        <v>80</v>
       </c>
       <c r="Z60" t="s" s="2">
-        <v>424</v>
+        <v>80</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>80</v>
@@ -8592,28 +8606,28 @@
         <v>80</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI60" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ60" t="s" s="2">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="AK60" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL60" t="s" s="2">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="AM60" t="s" s="2">
-        <v>290</v>
+        <v>189</v>
       </c>
       <c r="AN60" t="s" s="2">
         <v>80</v>
@@ -8621,10 +8635,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8641,59 +8655,57 @@
         <v>80</v>
       </c>
       <c r="I61" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J61" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K61" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="L61" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="N61" t="s" s="2">
         <v>426</v>
       </c>
-      <c r="L61" t="s" s="2">
+      <c r="O61" t="s" s="2">
         <v>427</v>
       </c>
-      <c r="M61" t="s" s="2">
+      <c r="P61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q61" s="2"/>
+      <c r="R61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X61" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="Y61" t="s" s="2">
         <v>428</v>
       </c>
-      <c r="N61" t="s" s="2">
+      <c r="Z61" t="s" s="2">
         <v>429</v>
       </c>
-      <c r="O61" t="s" s="2">
-        <v>430</v>
-      </c>
-      <c r="P61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q61" t="s" s="2">
-        <v>431</v>
-      </c>
-      <c r="R61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z61" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AA61" t="s" s="2">
         <v>80</v>
       </c>
@@ -8710,7 +8722,7 @@
         <v>80</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>78</v>
@@ -8719,7 +8731,7 @@
         <v>89</v>
       </c>
       <c r="AI61" t="s" s="2">
-        <v>432</v>
+        <v>80</v>
       </c>
       <c r="AJ61" t="s" s="2">
         <v>101</v>
@@ -8731,7 +8743,7 @@
         <v>107</v>
       </c>
       <c r="AM61" t="s" s="2">
-        <v>433</v>
+        <v>295</v>
       </c>
       <c r="AN61" t="s" s="2">
         <v>80</v>
@@ -8739,10 +8751,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8759,81 +8771,85 @@
         <v>80</v>
       </c>
       <c r="I62" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="J62" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>327</v>
+        <v>431</v>
       </c>
       <c r="L62" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="M62" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="N62" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="O62" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="M62" t="s" s="2">
+      <c r="P62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q62" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="N62" s="2"/>
-      <c r="O62" t="s" s="2">
+      <c r="R62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF62" t="s" s="2">
+        <v>430</v>
+      </c>
+      <c r="AG62" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH62" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI62" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="P62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q62" s="2"/>
-      <c r="R62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF62" t="s" s="2">
-        <v>434</v>
-      </c>
-      <c r="AG62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH62" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI62" t="s" s="2">
-        <v>80</v>
       </c>
       <c r="AJ62" t="s" s="2">
         <v>101</v>
@@ -8864,10 +8880,10 @@
       </c>
       <c r="E63" s="2"/>
       <c r="F63" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G63" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H63" t="s" s="2">
         <v>80</v>
@@ -8879,16 +8895,18 @@
         <v>80</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="L63" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="L63" t="s" s="2">
+      <c r="M63" t="s" s="2">
         <v>441</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" s="2"/>
+      <c r="O63" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
         <v>80</v>
       </c>
@@ -8939,7 +8957,7 @@
         <v>439</v>
       </c>
       <c r="AG63" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="AH63" t="s" s="2">
         <v>89</v>
@@ -8951,13 +8969,13 @@
         <v>101</v>
       </c>
       <c r="AK63" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL63" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AM63" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="AL63" t="s" s="2">
-        <v>444</v>
-      </c>
-      <c r="AM63" t="s" s="2">
-        <v>445</v>
       </c>
       <c r="AN63" t="s" s="2">
         <v>80</v>
@@ -8965,10 +8983,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -8976,10 +8994,10 @@
       </c>
       <c r="E64" s="2"/>
       <c r="F64" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H64" t="s" s="2">
         <v>80</v>
@@ -8991,20 +9009,16 @@
         <v>80</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>216</v>
+        <v>445</v>
       </c>
       <c r="L64" t="s" s="2">
+        <v>446</v>
+      </c>
+      <c r="M64" t="s" s="2">
         <v>447</v>
       </c>
-      <c r="M64" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="N64" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="O64" t="s" s="2">
-        <v>450</v>
-      </c>
+      <c r="N64" s="2"/>
+      <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
         <v>80</v>
       </c>
@@ -9028,13 +9042,13 @@
         <v>80</v>
       </c>
       <c r="X64" t="s" s="2">
-        <v>170</v>
+        <v>80</v>
       </c>
       <c r="Y64" t="s" s="2">
-        <v>451</v>
+        <v>80</v>
       </c>
       <c r="Z64" t="s" s="2">
-        <v>452</v>
+        <v>80</v>
       </c>
       <c r="AA64" t="s" s="2">
         <v>80</v>
@@ -9052,35 +9066,151 @@
         <v>80</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="AG64" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="AH64" t="s" s="2">
         <v>89</v>
       </c>
       <c r="AI64" t="s" s="2">
-        <v>408</v>
+        <v>80</v>
       </c>
       <c r="AJ64" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK64" t="s" s="2">
-        <v>80</v>
+        <v>448</v>
       </c>
       <c r="AL64" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="AM64" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="AN64" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="65" hidden="true">
+      <c r="A65" t="s" s="2">
+        <v>451</v>
+      </c>
+      <c r="B65" t="s" s="2">
+        <v>451</v>
+      </c>
+      <c r="C65" s="2"/>
+      <c r="D65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E65" s="2"/>
+      <c r="F65" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G65" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K65" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="L65" t="s" s="2">
+        <v>452</v>
+      </c>
+      <c r="M65" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="N65" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="O65" t="s" s="2">
+        <v>455</v>
+      </c>
+      <c r="P65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q65" s="2"/>
+      <c r="R65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X65" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="Y65" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="Z65" t="s" s="2">
+        <v>457</v>
+      </c>
+      <c r="AA65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF65" t="s" s="2">
+        <v>451</v>
+      </c>
+      <c r="AG65" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH65" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI65" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AJ65" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="AK65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL65" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="AM64" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="AN64" t="s" s="2">
+      <c r="AM65" t="s" s="2">
+        <v>458</v>
+      </c>
+      <c r="AN65" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN64">
+  <autoFilter ref="A1:AN65">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -9090,7 +9220,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI63">
+  <conditionalFormatting sqref="A2:AI64">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>